<commit_message>
feat(simulators): add guided vetting panels and NVIC simulator
</commit_message>
<xml_diff>
--- a/curriculum_progress_tracker.xlsx
+++ b/curriculum_progress_tracker.xlsx
@@ -136,7 +136,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -216,11 +216,60 @@
         <color rgb="00CBD5E1"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CBD5E1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CBD5E1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -306,6 +355,11 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -729,7 +783,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A4:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -741,9 +795,6 @@
     <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -814,7 +865,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
@@ -867,7 +917,6 @@
         <v/>
       </c>
     </row>
-    <row r="11"/>
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
@@ -913,7 +962,6 @@
         <v/>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
@@ -959,7 +1007,6 @@
         <v/>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
@@ -1069,7 +1116,6 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="1" t="inlineStr">
         <is>
@@ -1083,6 +1129,12 @@
           <t>Active Blockages &amp; Mentor Directive Actions</t>
         </is>
       </c>
+      <c r="B25" s="29" t="n"/>
+      <c r="C25" s="29" t="n"/>
+      <c r="D25" s="29" t="n"/>
+      <c r="E25" s="29" t="n"/>
+      <c r="F25" s="29" t="n"/>
+      <c r="G25" s="30" t="n"/>
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="10" t="inlineStr">
@@ -1090,8 +1142,22 @@
           <t>Sivaramireddy is executing exceptionally. Embedded Weeks 1-2 and C/Python Week 1 are in progress. Focus on making sure compiler flags are completely mastered this week. Ensure Mypy strict checks pass without 'Any' type bypasses inside the Python scripts.</t>
         </is>
       </c>
-    </row>
-    <row r="27" ht="20" customHeight="1"/>
+      <c r="B26" s="31" t="n"/>
+      <c r="C26" s="31" t="n"/>
+      <c r="D26" s="31" t="n"/>
+      <c r="E26" s="31" t="n"/>
+      <c r="F26" s="31" t="n"/>
+      <c r="G26" s="32" t="n"/>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="33" t="n"/>
+      <c r="B27" s="34" t="n"/>
+      <c r="C27" s="34" t="n"/>
+      <c r="D27" s="34" t="n"/>
+      <c r="E27" s="34" t="n"/>
+      <c r="F27" s="34" t="n"/>
+      <c r="G27" s="35" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="26">
     <mergeCell ref="D12"/>
@@ -1109,8 +1175,8 @@
     <mergeCell ref="B12"/>
     <mergeCell ref="C10"/>
     <mergeCell ref="C16"/>
+    <mergeCell ref="A25:G25"/>
     <mergeCell ref="E10"/>
-    <mergeCell ref="A25:G25"/>
     <mergeCell ref="D13"/>
     <mergeCell ref="E13"/>
     <mergeCell ref="C9"/>
@@ -1161,7 +1227,6 @@
       </c>
     </row>
     <row r="2"/>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="18" t="inlineStr">
         <is>
@@ -1231,11 +1296,11 @@
         </is>
       </c>
       <c r="E5" s="20" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="F5" s="11" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="G5" s="20" t="n">
@@ -1246,7 +1311,7 @@
       </c>
       <c r="I5" s="10" t="inlineStr">
         <is>
-          <t>Excellent repo setup and hook configurations.</t>
+          <t>Code compiled successfully, but overall systems explanation needs work.</t>
         </is>
       </c>
     </row>
@@ -2421,7 +2486,6 @@
       </c>
     </row>
     <row r="2"/>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="23" t="inlineStr">
         <is>
@@ -2917,7 +2981,6 @@
       </c>
     </row>
     <row r="2"/>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="24" t="inlineStr">
         <is>

</xml_diff>